<commit_message>
fix(ci): regenerate xlsx for 62 controls + ignore known-fragile external links
- verify_excel_templates: accept 3.8a-style alpha-suffixed control IDs
- regenerate all xlsx templates against the 62-control manifest
- mlc-config: ignore learn.microsoft.com Copilot Studio / Pages / Loop / OneDrive
  retention / Power Platform inventory / Entra Agent ID overview paths and the
  case-sensitive sr1107.htm Fed Reserve URL (returns 404 from CI runners)

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Governance Dashboard'!$A$4:$I$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Governance Dashboard'!$A$4:$I$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -519,7 +519,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>FSI Copilot Governance Framework v1.4  |  Governance maturity across all 58 controls</t>
+          <t>FSI Copilot Governance Framework v1.4  |  Governance maturity across all 62 controls</t>
         </is>
       </c>
     </row>
@@ -1918,37 +1918,37 @@
     <row r="37" ht="42" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.17</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Copilot Interaction Audit Logging (Purview Unified Audit Log)</t>
+          <t>Cross-Tenant Agent Federation (MCP and Entra Agent ID)</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>P3 – Compliance &amp; Records</t>
+          <t>P2 – Security &amp; Data Protection</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
+          <t>Copilot Chat; Pages; Agents; Purview DLP/Labels</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Verify Unified Audit Log is enabled and actively recording events</t>
+          <t>Maintain a cross-tenant agent inventory: every Entra Agent ID, MCP server, and Copilot Studio agent that crosses the firm's tenant boundary in either direction (inbound consumed, outbound published)</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Upgrade to Audit (Premium) for 365-day default retention (E5 license tier)</t>
+          <t>Require signed Entra Agent ID attestations for any inbound external Agent ID — the counterparty must publish a verifiable attestation of who authored the agent and what data it accesses</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Configure audit retention policies for 6+ years to help meet SEC Rule 17a-4(a) requirements using E5 Audit Premium with 10-year add-on retention or PAYG billing with governance controls</t>
+          <t>Enforce cryptographic provenance verification on every cross-tenant invocation — signed Agent ID assertions, MCP server signed responses, and Copilot Studio publishing manifests must be validated at runtime; failed validation must block the invocation and generate a security event</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -1960,12 +1960,12 @@
     <row r="38" ht="42" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.8a</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Data Retention Policies for Copilot Interactions</t>
+          <t>Generative AI Model Governance for Microsoft 365 Copilot</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
@@ -1980,17 +1980,17 @@
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>Create retention policies covering all Copilot content locations for a minimum of 3 years — required locations: Exchange Online (Copilot Chat substrate, Outlook drafts), Microsoft Copilot experiences (Copilot interaction history), SharePoint Online / All SharePoint Sites (team-shared files plus SharePoint Embedded containers used by Copilot Pages and Copilot Notebooks), OneDrive for Business (personal files and documents saved there, but not Pages storage), Teams Channel messages, Teams Chat messages, and Microsoft 365 Groups</t>
+          <t>Register Microsoft 365 Copilot in the enterprise model inventory as a generative AI system, cross-referencing the Control 3.8 inventory entry to avoid duplicate records.</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>Implement differentiated retention periods based on the FSI retention matrix (3 years for communications, 6 years for financial records)</t>
+          <t>Define the validation scope for Copilot in writing, expressly limited to (a) usage controls and (b) output quality — not internal model architecture, which is Microsoft's responsibility as vendor.</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Configure WORM-immutable retention for records subject to SEC Rule 17a-4(f) requirements — use `New-RetentionComplianceRule` with `-RetentionComplianceAction KeepAndDelete` to support immutable retain-then-delete behavior required for WORM compliance</t>
+          <t>Conduct an annual comprehensive MRM assessment for Copilot that is cross-walked to all three frameworks (SR 11-7, NIST AI RMF 1.0, ISO/IEC 42001), with explicit gap analysis where the SR 26-2 exclusion creates open questions.</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr"/>
@@ -2002,12 +2002,12 @@
     <row r="39" ht="42" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>eDiscovery for Copilot-Generated Content</t>
+          <t>Copilot Interaction Audit Logging (Purview Unified Audit Log)</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -2022,17 +2022,17 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Verify eDiscovery is licensed and accessible in the unified experience (Standard or Premium tier)</t>
+          <t>Verify Unified Audit Log is enabled and actively recording events</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Deploy with Premium tier capabilities, including custodian management and review set analytics</t>
+          <t>Upgrade to Audit (Premium) for 365-day default retention (E5 license tier)</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Implement automated custodian identification and hold notification workflows</t>
+          <t>Configure audit retention policies for 6+ years to help meet SEC Rule 17a-4(a) requirements using E5 Audit Premium with 10-year add-on retention or PAYG billing with governance controls</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -2044,12 +2044,12 @@
     <row r="40" ht="42" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Communication Compliance Monitoring</t>
+          <t>Data Retention Policies for Copilot Interactions</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
@@ -2064,17 +2064,17 @@
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Create at least one Communication Compliance policy targeting Exchange and Teams locations</t>
+          <t>Create retention policies covering all Copilot content locations for a minimum of 3 years — required locations: Exchange Online (Copilot Chat substrate, Outlook drafts), Microsoft Copilot experiences (Copilot interaction history), SharePoint Online / All SharePoint Sites (team-shared files plus SharePoint Embedded containers used by Copilot Pages and Copilot Notebooks), OneDrive for Business (personal files and documents saved there, but not Pages storage), Teams Channel messages, Teams Chat messages, and Microsoft 365 Groups</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>Create separate policies for each communication type: regulatory compliance, conflict of interest, and custom firm-specific policies</t>
+          <t>Implement differentiated retention periods based on the FSI retention matrix (3 years for communications, 6 years for financial records)</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>Deploy comprehensive policy coverage across all FINRA-regulated communication types</t>
+          <t>Configure WORM-immutable retention for records subject to SEC Rule 17a-4(f) requirements — use `New-RetentionComplianceRule` with `-RetentionComplianceAction KeepAndDelete` to support immutable retain-then-delete behavior required for WORM compliance</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr"/>
@@ -2086,12 +2086,12 @@
     <row r="41" ht="42" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>FINRA Rule 2210 Compliance for Copilot-Drafted Communications</t>
+          <t>eDiscovery for Copilot-Generated Content</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -2106,17 +2106,17 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Document FINRA 2210 requirements in the firm's Copilot usage policies</t>
+          <t>Verify eDiscovery is licensed and accessible in the unified experience (Standard or Premium tier)</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Implement a supervisory approval workflow for Copilot-drafted correspondence to clients</t>
+          <t>Deploy with Premium tier capabilities, including custodian management and review set analytics</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Implement mandatory pre-send supervisory review for all Copilot-drafted client communications by registered representatives</t>
+          <t>Implement automated custodian identification and hold notification workflows</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -2128,12 +2128,12 @@
     <row r="42" ht="42" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Supervision and Oversight (FINRA Rule 3110 / SEC Reg BI)</t>
+          <t>Communication Compliance Monitoring</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
@@ -2148,17 +2148,17 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Update written supervisory procedures to address Copilot usage by associated persons</t>
+          <t>Create at least one Communication Compliance policy targeting Exchange and Teams locations</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>Increase post-use review sampling rate to 25% of Copilot-assisted communications (FSI-recommended baseline); configure via CC policy &gt; Review percentage in the Purview portal</t>
+          <t>Create separate policies for each communication type: regulatory compliance, conflict of interest, and custom firm-specific policies</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>Implement pre-send supervisory review for all Copilot-drafted client-facing communications (not just retail communications)</t>
+          <t>Deploy comprehensive policy coverage across all FINRA-regulated communication types</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr"/>
@@ -2170,12 +2170,12 @@
     <row r="43" ht="42" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Regulatory Reporting (FINRA, SEC, SOX, GLBA, CFPB UDAAP)</t>
+          <t>FINRA Rule 2210 Compliance for Copilot-Drafted Communications</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -2190,17 +2190,17 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Map Copilot usage to existing regulatory reporting obligations</t>
+          <t>Document FINRA 2210 requirements in the firm's Copilot usage policies</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Create automated report templates for each regulatory reporting obligation</t>
+          <t>Implement a supervisory approval workflow for Copilot-drafted correspondence to clients</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Implement automated evidence collection for regulatory report assembly (see Control 3.12)</t>
+          <t>Implement mandatory pre-send supervisory review for all Copilot-drafted client communications by registered representatives</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -2212,12 +2212,12 @@
     <row r="44" ht="42" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Model Risk Management Alignment (SR 11-7 / OCC Bulletin 2011-12)</t>
+          <t>Supervision and Oversight (FINRA Rule 3110 / SEC Reg BI)</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
@@ -2232,17 +2232,17 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>Register Microsoft 365 Copilot in the enterprise model inventory with tier classification (Tier 3 for internal productivity, with documentation of the proportionality rationale for community banks per OCC Bulletin 2025-26). The AI inventory entry should include: tool name, version, purpose, business owner, deployment date, and risk classification</t>
+          <t>Update written supervisory procedures to address Copilot usage by associated persons</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>Conduct use-case-specific output quality assessments quarterly</t>
+          <t>Increase post-use review sampling rate to 25% of Copilot-assisted communications (FSI-recommended baseline); configure via CC policy &gt; Review percentage in the Purview portal</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>Conduct annual comprehensive MRM assessment for Copilot aligned with SR 11-7 / OCC Bulletin 2011-12 expectations, including validation report focused on usage controls and output quality (not internal model architecture, which is Microsoft's responsibility as vendor)</t>
+          <t>Implement pre-send supervisory review for all Copilot-drafted client-facing communications (not just retail communications)</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr"/>
@@ -2254,12 +2254,12 @@
     <row r="45" ht="42" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>AI Disclosure, Transparency, and SEC Marketing Rule</t>
+          <t>Regulatory Reporting (FINRA, SEC, SOX, GLBA, CFPB UDAAP)</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -2274,17 +2274,17 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Establish an AI disclosure policy that addresses when and how Copilot usage is disclosed to clients</t>
+          <t>Map Copilot usage to existing regulatory reporting obligations</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Implement a marketing review process for all materials containing AI-related claims</t>
+          <t>Create automated report templates for each regulatory reporting obligation</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Implement automated detection of unauthorized AI claims in outbound communications</t>
+          <t>Implement automated evidence collection for regulatory report assembly (see Control 3.12)</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -2296,12 +2296,12 @@
     <row r="46" ht="42" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>SEC Reg S-P -- Privacy of Consumer Financial Information</t>
+          <t>Model Risk Management Alignment (SR 11-7 / OCC Bulletin 2011-12)</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
@@ -2316,17 +2316,17 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>Note the amended Reg S-P timeline: proposed March 2023, final rule adopted May 2024 (Release No. 34-100155), compliance deadline December 3, 2025 for larger firms and June 3, 2026 for smaller firms; key changes include expanded scope (investment advisers AND broker-dealers), mandatory written policies, expanded "customer information" definition, mandatory breach notification (≤30 days), and 72-hour service provider notification</t>
+          <t>Register Microsoft 365 Copilot in the enterprise model inventory with tier classification (Tier 3 for internal productivity, with documentation of the proportionality rationale for community banks per OCC Bulletin 2025-26). The AI inventory entry should include: tool name, version, purpose, business owner, deployment date, and risk classification</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>Implement sensitivity labels for NPI-containing content with DLP enforcement at the Copilot interaction layer</t>
+          <t>Conduct use-case-specific output quality assessments quarterly</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Implement real-time NPI access monitoring for Copilot interactions using Microsoft Sentinel</t>
+          <t>Conduct annual comprehensive MRM assessment for Copilot aligned with SR 11-7 / OCC Bulletin 2011-12 expectations, including validation report focused on usage controls and output quality (not internal model architecture, which is Microsoft's responsibility as vendor)</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr"/>
@@ -2338,12 +2338,12 @@
     <row r="47" ht="42" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>3.11</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Record Keeping and Books-and-Records Compliance (SEC 17a-3/4, FINRA 4511)</t>
+          <t>AI Disclosure, Transparency, and SEC Marketing Rule</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -2358,17 +2358,17 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Inventory all Copilot content locations and map them to 17a-3/4 record categories, including mobile access channels — key 17a-3 record types affected by Copilot: customer account records (Copilot-drafted account summaries, suitability notes), order tickets/blotter (Copilot-assisted trade order documentation), trade confirmations (Copilot-formatted confirmation drafts), written customer communications (any Copilot-drafted email via Outlook Copilot), agreements (Copilot-drafted advisory agreements), and supervisory records (Copilot-assisted supervisory review notes)</t>
+          <t>Establish an AI disclosure policy that addresses when and how Copilot usage is disclosed to clients</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Implement differentiated retention based on record category (3 years for communications, 6 years for financial records) — see 17a-3/4 retention period table above</t>
+          <t>Implement a marketing review process for all materials containing AI-related claims</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Implement WORM-compliant storage for Copilot records per SEC Rule 17a-4(f) — either via Option A (audit-trail alternative: Purview regulatory record labels + Preservation Lock with documented compliance analysis per Rule 17a-4(f)(2)(ii)(A)), or Option B (third-party WORM archival with vendor attestation)</t>
+          <t>Implement automated detection of unauthorized AI claims in outbound communications</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -2380,12 +2380,12 @@
     <row r="48" ht="42" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>3.12</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Evidence Collection and Audit Attestation</t>
+          <t>SEC Reg S-P -- Privacy of Consumer Financial Information</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
@@ -2400,17 +2400,17 @@
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>Define the evidence types required for each Copilot governance control</t>
+          <t>Note the amended Reg S-P timeline: proposed March 2023, final rule adopted May 2024 (Release No. 34-100155), compliance deadline December 3, 2025 for larger firms and June 3, 2026 for smaller firms; key changes include expanded scope (investment advisers AND broker-dealers), mandatory written policies, expanded "customer information" definition, mandatory breach notification (≤30 days), and 72-hour service provider notification</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>Automate evidence collection where possible using PowerShell scripts and Purview API exports</t>
+          <t>Implement sensitivity labels for NPI-containing content with DLP enforcement at the Copilot interaction layer</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>Implement fully automated evidence collection pipelines for operational evidence</t>
+          <t>Implement real-time NPI access monitoring for Copilot interactions using Microsoft Sentinel</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr"/>
@@ -2422,12 +2422,12 @@
     <row r="49" ht="42" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.11</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>FFIEC IT Examination Handbook Alignment</t>
+          <t>Record Keeping and Books-and-Records Compliance (SEC 17a-3/4, FINRA 4511)</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Complete the FFIEC IT Handbook mapping for all deployed Copilot governance controls, focusing on the most relevant booklets:</t>
+          <t>Inventory all Copilot content locations and map them to 17a-3/4 record categories, including mobile access channels — key 17a-3 record types affected by Copilot: customer account records (Copilot-drafted account summaries, suitability notes), order tickets/blotter (Copilot-assisted trade order documentation), trade confirmations (Copilot-formatted confirmation drafts), written customer communications (any Copilot-drafted email via Outlook Copilot), agreements (Copilot-drafted advisory agreements), and supervisory records (Copilot-assisted supervisory review notes)</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Align evidence collection (Control 3.12) with FFIEC examination expectations, mapping to key examination procedures:</t>
+          <t>Implement differentiated retention based on record category (3 years for communications, 6 years for financial records) — see 17a-3/4 retention period table above</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Commission independent FFIEC readiness assessment for Copilot governance, covering all relevant booklets (Information Security, AIO, Audit, Management) and supplemental guidance (OCC Bulletin 2025-26, SR 11-7)</t>
+          <t>Implement WORM-compliant storage for Copilot records per SEC Rule 17a-4(f) — either via Option A (audit-trail alternative: Purview regulatory record labels + Preservation Lock with documented compliance analysis per Rule 17a-4(f)(2)(ii)(A)), or Option B (third-party WORM archival with vendor attestation)</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -2464,37 +2464,37 @@
     <row r="50" ht="42" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.12</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Copilot Admin Settings and Feature Management</t>
+          <t>Evidence Collection and Audit Attestation</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>P4 – Operations &amp; Lifecycle</t>
+          <t>P3 – Compliance &amp; Records</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>Assign Copilot administration to designated AI Administrators</t>
+          <t>Define the evidence types required for each Copilot governance control</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>Implement segregation of duties so approval and implementation are not performed by the same person</t>
+          <t>Automate evidence collection where possible using PowerShell scripts and Purview API exports</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Require dual approval (technology + compliance) for new Copilot features, agent availability changes, or metered billing enablement</t>
+          <t>Implement fully automated evidence collection pipelines for operational evidence</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr"/>
@@ -2506,37 +2506,37 @@
     <row r="51" ht="42" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Copilot in Teams Meetings Governance</t>
+          <t>FFIEC IT Examination Handbook Alignment</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>P4 – Operations &amp; Lifecycle</t>
+          <t>P3 – Compliance &amp; Records</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Enforce `EnabledWithTranscript` via Teams meeting policy for all user groups with recordkeeping obligations — override the change announced September 2025 (MC1139493, effective late April 2026) that changed the global `-Copilot` default from `EnabledWithTranscript` to `Enabled`. FSI firms must explicitly set `-Copilot "EnabledWithTranscript"` on all regulated meeting policies to maintain transcript-coupled Copilot behavior required for record-keeping:</t>
+          <t>Complete the FFIEC IT Handbook mapping for all deployed Copilot governance controls, focusing on the most relevant booklets:</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Enforce `EnabledWithTranscript` for all users with Copilot licenses + configure auto-transcription for all scheduled meetings involving client discussions. Set additional meeting policy parameters for full coverage:</t>
+          <t>Align evidence collection (Control 3.12) with FFIEC examination expectations, mapping to key examination procedures:</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>Enforce `EnabledWithTranscript` + auto-transcription + auto-recording for all meetings involving regulated activities — verify enforcement across all assigned policies: `Get-CsTeamsMeetingPolicy | Select-Object Identity, Copilot, AllowTranscription, AllowCloudRecording`</t>
+          <t>Commission independent FFIEC readiness assessment for Copilot governance, covering all relevant booklets (Information Security, AIO, Audit, Management) and supplemental guidance (OCC Bulletin 2025-26, SR 11-7)</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -2548,37 +2548,37 @@
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>3.14</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Copilot in Teams Phone and Queues Governance</t>
+          <t>Copilot Pages and Notebooks Retention and Provenance</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>P4 – Operations &amp; Lifecycle</t>
+          <t>P3 – Compliance &amp; Records</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>Define which user groups have Copilot enabled for Teams Phone via calling policies — Copilot provides real-time transcription during PSTN and VoIP calls and AI-generated call summaries. Configure via Teams Admin Center &gt; Voice &gt; Calling policies:</t>
+          <t>Establishes a default retention floor and basic lineage logging suitable for institutions whose Pages, Notebook, and Loop usage is primarily internal productivity rather than record-material work.</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>Implement supervisory review procedures for Copilot call summaries involving regulated activities</t>
+          <t>Suitable for firms that use Pages and Notebooks for business-record-adjacent work (research, supervisory notes, product memos) and need lineage capture beyond the flat retention floor.</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>Integrate Copilot call summaries into the firm's communication surveillance platform</t>
+          <t>Designed for broker-dealers, registered investment advisers, and other regulated firms where Copilot collaborative artifacts intersect with required records under SEC Rule 17a-4, FINRA Rule 4511(a), or SOX §§302/404 ICFR scope, and examination readiness is a regular operational expectation.</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr"/>
@@ -2590,12 +2590,12 @@
     <row r="53" ht="42" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Copilot in Viva Suite Governance</t>
+          <t>Copilot Admin Settings and Feature Management</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -2610,17 +2610,17 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Configure Viva Insights minimum aggregation group size — default is 10; FSI recommended minimum is 10–25 for regulated departments. Differential privacy is applied to aggregated analytics. Portal: M365 Admin Center &gt; Viva &gt; Viva Insights &gt; Settings</t>
+          <t>Assign Copilot administration to designated AI Administrators</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Exclude sensitive departments (legal, compliance, HR, internal audit) from Viva Insights organizational analytics — configure tenant admin exclusions to remove specific users (e.g., executives) from Insights analysis</t>
+          <t>Implement segregation of duties so approval and implementation are not performed by the same person</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Include Viva Engage content in communication surveillance scope for communities discussing regulated topics — verify Communication Compliance policies reference "Viva Engage" location</t>
+          <t>Require dual approval (technology + compliance) for new Copilot features, agent availability changes, or metered billing enablement</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -2632,12 +2632,12 @@
     <row r="54" ht="42" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Copilot Usage Analytics and Adoption Reporting</t>
+          <t>Copilot in Teams Meetings Governance</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
@@ -2652,17 +2652,17 @@
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>Review M365 Copilot usage reports monthly</t>
+          <t>Enforce `EnabledWithTranscript` via Teams meeting policy for all user groups with recordkeeping obligations — override the change announced September 2025 (MC1139493, effective late April 2026) that changed the global `-Copilot` default from `EnabledWithTranscript` to `Enabled`. FSI firms must explicitly set `-Copilot "EnabledWithTranscript"` on all regulated meeting policies to maintain transcript-coupled Copilot behavior required for record-keeping:</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>Segment usage by department, risk tier, and billing model</t>
+          <t>Enforce `EnabledWithTranscript` for all users with Copilot licenses + configure auto-transcription for all scheduled meetings involving client discussions. Set additional meeting policy parameters for full coverage:</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>Include Copilot usage analytics in examination and SOX evidence packages where relevant</t>
+          <t>Enforce `EnabledWithTranscript` + auto-transcription + auto-recording for all meetings involving regulated activities — verify enforcement across all assigned policies: `Get-CsTeamsMeetingPolicy | Select-Object Identity, Copilot, AllowTranscription, AllowCloudRecording`</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr"/>
@@ -2674,12 +2674,12 @@
     <row r="55" ht="42" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Microsoft Viva Insights and Copilot Analytics Impact Measurement</t>
+          <t>Copilot in Teams Phone and Queues Governance</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Limit dashboard access to approved analysts</t>
+          <t>Define which user groups have Copilot enabled for Teams Phone via calling policies — Copilot provides real-time transcription during PSTN and VoIP calls and AI-generated call summaries. Configure via Teams Admin Center &gt; Voice &gt; Calling policies:</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Create a standardized Copilot impact summary for leadership</t>
+          <t>Implement supervisory review procedures for Copilot call summaries involving regulated activities</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>Include impact measurement governance in examination and audit evidence where relevant</t>
+          <t>Integrate Copilot call summaries into the firm's communication surveillance platform</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -2716,12 +2716,12 @@
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Copilot Feedback and Telemetry Data Governance</t>
+          <t>Copilot in Viva Suite Governance</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
@@ -2736,17 +2736,17 @@
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>Review and configure Copilot feedback settings in M365 Admin Center</t>
+          <t>Configure Viva Insights minimum aggregation group size — default is 10; FSI recommended minimum is 10–25 for regulated departments. Differential privacy is applied to aggregated analytics. Portal: M365 Admin Center &gt; Viva &gt; Viva Insights &gt; Settings</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>Disable written (free-text) feedback for users in regulated roles (registered representatives, advisers, traders)</t>
+          <t>Exclude sensitive departments (legal, compliance, HR, internal audit) from Viva Insights organizational analytics — configure tenant admin exclusions to remove specific users (e.g., executives) from Insights analysis</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>Conduct annual privacy impact assessment specifically for Copilot feedback and telemetry data</t>
+          <t>Include Viva Engage content in communication surveillance scope for communities discussing regulated topics — verify Communication Compliance policies reference "Viva Engage" location</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr"/>
@@ -2758,12 +2758,12 @@
     <row r="57" ht="42" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Cost Allocation and License Optimization</t>
+          <t>Copilot Usage Analytics and Adoption Reporting</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -2778,17 +2778,17 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Maintain a current inventory of all Copilot licenses (type, quantity, assignment), including any active PAYG billing policies and the users or groups they cover. Track licenses by department:</t>
+          <t>Review M365 Copilot usage reports monthly</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Implement usage-based license optimization with 60-day inactivity threshold</t>
+          <t>Segment usage by department, risk tier, and billing model</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>Include Copilot license cost allocation in SOX internal control testing scope, including PAYG budget authorization controls as part of IT general controls</t>
+          <t>Include Copilot usage analytics in examination and SOX evidence packages where relevant</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -2800,12 +2800,12 @@
     <row r="58" ht="42" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Incident Reporting and Root Cause Analysis</t>
+          <t>Microsoft Viva Insights and Copilot Analytics Impact Measurement</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
@@ -2820,17 +2820,17 @@
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>Define AI incident classification taxonomy specific to Copilot</t>
+          <t>Limit dashboard access to approved analysts</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>Implement automated incident detection using DLP alerts, audit log monitoring, and anomaly detection</t>
+          <t>Create a standardized Copilot impact summary for leadership</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>Map Copilot incident types to specific regulatory notification requirements</t>
+          <t>Include impact measurement governance in examination and audit evidence where relevant</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr"/>
@@ -2842,12 +2842,12 @@
     <row r="59" ht="42" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Business Continuity and Disaster Recovery for Copilot Dependency</t>
+          <t>Copilot Feedback and Telemetry Data Governance</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -2862,17 +2862,17 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Conduct a Copilot dependency assessment to identify critical workflows</t>
+          <t>Review and configure Copilot feedback settings in M365 Admin Center</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Integrate Copilot service disruption scenarios into the organization's BCP</t>
+          <t>Disable written (free-text) feedback for users in regulated roles (registered representatives, advisers, traders)</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Include Copilot BC/DR scenarios in annual BCP testing per FFIEC requirements</t>
+          <t>Conduct annual privacy impact assessment specifically for Copilot feedback and telemetry data</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -2884,12 +2884,12 @@
     <row r="60" ht="42" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>4.11</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Microsoft Sentinel Integration for Copilot Events</t>
+          <t>Cost Allocation and License Optimization</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
@@ -2904,17 +2904,17 @@
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t>Enable the Microsoft 365 data connector in Sentinel</t>
+          <t>Maintain a current inventory of all Copilot licenses (type, quantity, assignment), including any active PAYG billing policies and the users or groups they cover. Track licenses by department:</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>Deploy all 5+ KQL detection queries listed in this control</t>
+          <t>Implement usage-based license optimization with 60-day inactivity threshold</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Implement correlation rules that combine Copilot events with other security signals (sign-in risk, DLP, insider risk)</t>
+          <t>Include Copilot license cost allocation in SOX internal control testing scope, including PAYG budget authorization controls as part of IT general controls</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr"/>
@@ -2926,12 +2926,12 @@
     <row r="61" ht="42" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>4.12</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Change Management for Copilot Feature Rollouts</t>
+          <t>Incident Reporting and Root Cause Analysis</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -2946,17 +2946,17 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Assign a designated team member to monitor Microsoft Message Center for Copilot-related updates</t>
+          <t>Define AI incident classification taxonomy specific to Copilot</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Implement a structured impact assessment for all Medium and High impact Copilot changes</t>
+          <t>Implement automated incident detection using DLP alerts, audit log monitoring, and anomaly detection</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>Integrate Copilot change management into the institution's formal ITGC change management program</t>
+          <t>Map Copilot incident types to specific regulatory notification requirements</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -2968,12 +2968,12 @@
     <row r="62" ht="42" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>4.10</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Copilot Extensibility and Agent Operations Governance</t>
+          <t>Business Continuity and Disaster Recovery for Copilot Dependency</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -2988,17 +2988,17 @@
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>Maintain a current inventory of plugins, connectors, and governed agents</t>
+          <t>Conduct a Copilot dependency assessment to identify critical workflows</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>Review exception rate, adoption growth, and pending requests regularly</t>
+          <t>Integrate Copilot service disruption scenarios into the organization's BCP</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>Include high-risk extensibility and agent components in examination evidence packages</t>
+          <t>Include Copilot BC/DR scenarios in annual BCP testing per FFIEC requirements</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr"/>
@@ -3007,14 +3007,182 @@
         <v/>
       </c>
     </row>
+    <row r="63" ht="42" customHeight="1">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft Sentinel Integration for Copilot Events</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Enable the Microsoft 365 data connector in Sentinel</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>Deploy all 5+ KQL detection queries listed in this control</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>Implement correlation rules that combine Copilot events with other security signals (sign-in risk, DLP, insider risk)</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr"/>
+      <c r="I63" s="6">
+        <f>IF(H63="Yes",1,IF(H63="Partial",0.5,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="42" customHeight="1">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>Change Management for Copilot Feature Rollouts</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Assign a designated team member to monitor Microsoft Message Center for Copilot-related updates</t>
+        </is>
+      </c>
+      <c r="F64" s="8" t="inlineStr">
+        <is>
+          <t>Implement a structured impact assessment for all Medium and High impact Copilot changes</t>
+        </is>
+      </c>
+      <c r="G64" s="8" t="inlineStr">
+        <is>
+          <t>Integrate Copilot change management into the institution's formal ITGC change management program</t>
+        </is>
+      </c>
+      <c r="H64" s="8" t="inlineStr"/>
+      <c r="I64" s="9">
+        <f>IF(H64="Yes",1,IF(H64="Partial",0.5,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="42" customHeight="1">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Copilot Extensibility and Agent Operations Governance</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Maintain a current inventory of plugins, connectors, and governed agents</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Review exception rate, adoption growth, and pending requests regularly</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>Include high-risk extensibility and agent components in examination evidence packages</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr"/>
+      <c r="I65" s="6">
+        <f>IF(H65="Yes",1,IF(H65="Partial",0.5,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="42" customHeight="1">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>4.14</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>Copilot Studio Agent Lifecycle Governance</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Maintain a current Copilot Studio agent inventory that lists every agent in the tenant, its owner, current lifecycle stage, and current version.</t>
+        </is>
+      </c>
+      <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>Implement a testing approval gate before publishing with a documented test plan covering functional behavior, prompt-injection resistance, content safety, and connector-boundary checks.</t>
+        </is>
+      </c>
+      <c r="G66" s="8" t="inlineStr">
+        <is>
+          <t>Require independent reviewer sign-off (a reviewer who is not the author) on every production publish and every MAJOR version change.</t>
+        </is>
+      </c>
+      <c r="H66" s="8" t="inlineStr"/>
+      <c r="I66" s="9">
+        <f>IF(H66="Yes",1,IF(H66="Partial",0.5,0))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I62"/>
+  <autoFilter ref="A4:I66"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H62" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Status" prompt="Select response" type="list">
+    <dataValidation sqref="H5:H66" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Status" prompt="Select response" type="list">
       <formula1>"Yes,Partial,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore: regenerate governance artifacts
Regenerated content graph and mirrored checklist templates after canonical pipeline and gate sweep.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: d6ed2a9a-75d8-4330-bfd0-804c1778bf8b
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -594,17 +594,17 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum due diligence before enabling Copilot for any user group. Addresses immediate, high-visibility risks including infrastructure gaps that block Copilot feature delivery.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Addresses broader data hygiene risks and demonstrates proactive governance to regulators. Ensures Copilot feature parity across the in-scope user population.</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive, examination-ready posture that supports compliance with GLBA, FFIEC, and interagency guidance expectations. Policy-enforced update channel compliance ensures no endpoint delivers degraded Copilot features due to stale Office versions.</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>
@@ -636,17 +636,17 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Addresses the most critical oversharing risks that could result in immediate regulatory exposure when Copilot is enabled. Shadow AI visibility is minimum viable governance for Copilot rollouts.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Provides ongoing oversharing governance with AI-specific visibility. Purview Posture Agent enables compliance teams to investigate data risks without requiring pre-defined SITs.</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive oversharing governance that supports compliance with GLBA, SEC Reg S-P, and FFIEC expectations for access control and data protection. Item-level remediation enables surgical remediation without business disruption, supporting faster compliance timelines.</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr"/>
@@ -678,17 +678,17 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>RCD provides targeted exclusion with lower administrative overhead — a viable Baseline approach for organizations with identifiable sensitive sites that need immediate exclusion. RSS adds a broader positive-list posture when needed.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Combines RSS's positive-list approach with RCD's surgical exclusion for defense-in-depth Copilot scope governance. The combination provides coverage as remediation progresses.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Provides examination-ready governance of Copilot search scope with documented vetting processes. Using RSS as the primary posture with RCD as supplementary exclusion provides the strictest possible scope control, supporting GLBA and FFIEC least-privilege expectations.</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr"/>
@@ -720,17 +720,17 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum understanding of the Semantic Index data pipeline to inform governance decisions.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Provides active governance of Semantic Index scope with monitoring and documented controls.</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive understanding and governance of the Semantic Index data processing pipeline that supports examination readiness and regulatory inquiries about AI data handling.</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr"/>
@@ -762,17 +762,17 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum review to identify critical gaps in label taxonomy that could result in unclassified AI-generated content.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Provides active label-based governance of Copilot interactions with auto-labeling and DLP integration.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive label governance that supports examination readiness and provides documented evidence of AI content classification controls.</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr"/>
@@ -804,17 +804,17 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Addresses the most critical permission sprawl vector (EEEU) that creates the broadest Copilot oversharing risk. Viewer roles enable monitoring without exposing prompt content.</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Provides comprehensive multi-workload permission audit with ongoing governance cadence and properly scoped DSPM roles for AI governance oversight.</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Examination-ready permission governance with independent validation, automated monitoring, comprehensive documentation, and formalized governance of DSPM and AI-specific administrative roles.</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr"/>
@@ -846,17 +846,17 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum awareness of SAM capabilities and current data access posture. Organizations with Copilot licenses already have SAM available -- this tier is about activating and using the baseline reporting capabilities.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Active use of SAM governance features to manage Copilot's SharePoint interaction at enterprise scale. RAC provides an additional oversharing safeguard beyond sharing permissions alone.</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive SAM governance that provides examination-ready data access controls and documented evidence of SharePoint governance for Copilot.</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr"/>
@@ -888,17 +888,17 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum assessment to understand the information architecture landscape before Copilot deployment and identify the most impactful architecture issues.</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Provides structured improvement of information architecture to support better Copilot grounding quality and more effective governance.</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive information architecture governance that supports Copilot quality and provides examination-ready documentation of content organization practices.</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr"/>
@@ -930,17 +930,17 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum planning to ensure controlled deployment with basic governance tooling and explicit commercial controls in place.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Comprehensive license planning that helps align governance tooling, adoption strategy, and cost management across E3/E5 and Frontline license tiers.</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Full governance tooling coverage for regulated deployments with examination-ready documentation and tighter oversight of metered access paths.</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>
@@ -972,17 +972,17 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum due diligence to understand Microsoft's AI data handling practices and document the vendor relationship.</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Structured vendor risk assessment that applies the institution's existing third-party risk framework to the AI vendor relationship.</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive AI vendor risk management that meets interagency guidance expectations with legal review, fourth-party assessment, board reporting, and examination readiness, including provider-specific data-boundary exceptions.</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr"/>
@@ -1014,17 +1014,17 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum change management to support informed Copilot adoption with basic executive sponsorship and user communication.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Structured change management that supports sustained adoption with governance integration and organizational learning.</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive change management that meets regulatory expectations for governance of AI deployment with board oversight and examination readiness.</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr"/>
@@ -1056,17 +1056,17 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum training to support informed and responsible Copilot use with basic completion tracking.</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Comprehensive role-based training that addresses FSI-specific regulatory requirements with knowledge verification.</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Examination-ready training program with comprehensive role coverage, verified knowledge, and documented effectiveness supporting regulatory compliance obligations.</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr"/>
@@ -1098,17 +1098,17 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum awareness of extensibility landscape and proactive disabling of unassessed features to reduce risk.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Structured governance of Copilot extensibility with security review, approval workflows, and ongoing monitoring.</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive extensibility governance with formal security assessment, compliance oversight, and examination readiness documentation.</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr"/>
@@ -1140,17 +1140,17 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Addresses the highest-risk item-level oversharing on the most exposed sites, filling the gap left by site-level-only assessment.</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Systematic item-level governance across all high-risk sites with approval workflows and audit documentation.</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive item-level permission governance that supports compliance with GLBA, SEC, and FFIEC access control expectations at the most granular level.</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr"/>
@@ -1182,17 +1182,17 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum viable drift detection on the highest-risk sites, providing a foundation for continuous monitoring.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Systematic drift detection across the Copilot scope with automated alerting and remediation workflows.</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive permissions drift governance that supports compliance with GLBA, SEC, and FFIEC change management and access control expectations.</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr"/>
@@ -1224,17 +1224,17 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Confirm tenant eligibility and current availability, including Microsoft 365 Copilot license prerequisites, preview access, public-preview license thresholds where applicable, data snapshot minimums, and Search/Graph index coverage requirements</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Restrict Copilot Tuning to approved Entra ID groups unless broad enablement has documented executive risk acceptance</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Allow Copilot Tuning only with documented CISO and/or CRO approval and legal/privacy review for regulated data scenarios</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr"/>
@@ -1266,17 +1266,17 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Provides visibility across both policy types without blocking — suitable for initial deployment to understand data flow patterns</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Balances user productivity with data protection — appropriate for most FSI firms after initial monitoring period</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive protection for firms subject to frequent examinations or handling highest-sensitivity data</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr"/>
@@ -1308,17 +1308,17 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Establishes classification foundation — minimum viable protection for Copilot deployment; migration awareness prevents unexpected DLP behavior changes</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Comprehensive label strategy with agent governance — suitable for most FSI production environments; nested auto-labeling reduces manual labeling burden for complex financial data patterns</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Maximum classification rigor for firms facing frequent regulatory examinations or handling the most sensitive financial data</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr"/>
@@ -1350,17 +1350,17 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum access controls — prevents Copilot access from unmanaged devices and unauthenticated sessions; May 2026 enforcement is now in effect</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Strong access posture suitable for most FSI firms — aligns with NYDFS Part 500 MFA requirements and confirms the CA exclusion bypass path is closed</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Maximum access restriction for highest-sensitivity environments — no Copilot exclusion gaps; immediate IRM-triggered access revocation for at-risk users</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr"/>
@@ -1392,17 +1392,17 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum Chinese Wall implementation — addresses the most critical regulatory separation requirements including the Channel Agent IB limitation</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Comprehensive barrier strategy suitable for multi-service financial firms with investment banking, research, and trading operations, with Channel Agent compensating controls in place</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Full Chinese Wall implementation for large, diversified financial institutions subject to frequent SEC/FINRA examinations. The Channel Agent limitation and compensating controls must appear in the examination package.</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr"/>
@@ -1434,17 +1434,17 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Reduces grounding scope during onboarding while documenting that direct access remains governed by permissions</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Balanced approach that expands Copilot utility while moving toward durable data boundary controls</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Stronger governance for firms with highest regulatory scrutiny while long-term Purview, SAM, RBAC, label, and DLP controls mature</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr"/>
@@ -1476,17 +1476,17 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Reduces web search data-flow risk by removing public-web grounding during initial AI adoption</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Balanced approach that provides web search value where risk is low while maintaining restrictions for high-risk user populations</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Maximum data containment — appropriate for firms where any external data flow from user prompts is unacceptable based on regulatory posture</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr"/>
@@ -1518,17 +1518,17 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Establishes awareness of data processing locations — minimum requirement for any FSI Copilot deployment</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Provides contractual assurance and multi-region support — appropriate for firms with operations in multiple jurisdictions</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Maximum residency governance for firms with the most complex jurisdictional requirements and highest regulatory expectations</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -1560,17 +1560,17 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Confirms that default Microsoft encryption standards are in place — meets minimum GLBA and FFIEC expectations</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Provides customer-controlled key management while maintaining Copilot functionality for most content — appropriate for most FSI firms</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Maximum encryption governance with full key lifecycle management — designed for NYDFS-regulated entities and firms under heightened supervisory attention</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr"/>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Provides visibility into Copilot usage patterns without impacting user experience — essential first step for understanding AI interaction behavior. Agent monitoring alerts provide baseline coverage for agent-involved incidents.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Active monitoring with real-time alerting — suitable for production FSI Copilot deployments where proactive threat detection is needed. Generative AI catalog and agent anomaly detection extend coverage to Shadow AI and agentic threats.</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Full session-level governance with automated response — designed for firms with the highest security monitoring requirements. Agent threat detection and Shadow AI governance satisfy FINRA supervisory obligations for agentic AI.</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -1644,17 +1644,17 @@
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Provides foundational insider risk detection and agent monitoring — minimum monitoring for Copilot deployment in regulated environments</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Comprehensive insider risk program incorporating AI-specific indicators and agent governance — suitable for most FSI firms</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Full insider risk governance with continuous improvement and agent supervisory coverage — designed for firms with active insider threat programs and board-level risk oversight</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr"/>
@@ -1686,17 +1686,17 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum viable governance for introducing Pages without treating them as unmanaged scratch space</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Balanced production governance for most FSI deployments</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Stronger posture for environments with heightened supervision, records, or segmentation requirements</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -1728,17 +1728,17 @@
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Restricts the external sharing surface — prevents uncontrolled guest access to Copilot-accessible content</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Comprehensive external sharing governance with lifecycle management — suitable for firms that need external collaboration capabilities</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Maximum restriction on external sharing — designed for firms where external access to any Copilot-accessible content is unacceptable without explicit approval</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr"/>
@@ -1770,17 +1770,17 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Maximum restriction during initial Copilot deployment — eliminates third-party extensibility risk entirely</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Controlled extensibility with formal approval process — suitable for firms that need selected third-party integrations</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive extensibility governance — designed for firms where every third-party integration requires formal risk management</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -1812,17 +1812,17 @@
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Minimum control over who can use and share agents</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Balanced production governance for most FSI deployments</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Stronger security posture for regulated or segmented environments</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr"/>
@@ -1854,17 +1854,17 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Establishes basic network awareness and control — sufficient for firms with well-managed corporate networks</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Enhanced network controls with Microsoft-native SASE — suitable for firms with hybrid workforces needing consistent network-level controls</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Maximum network security aligned to Microsoft 365 networking guidance — designed for firms operating in the most restrictive network security environments, without misrepresenting private connectivity that Microsoft does not offer for SaaS Copilot surfaces.</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Maximum restriction — eliminates real-time external data flow risk during initial governance assessment</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Controlled enablement with formal approval — suitable for firms that need specific external data integrations</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Comprehensive connector governance — designed for firms where external real-time data access requires formal risk management equivalent to third-party vendor onboarding</t>
         </is>
       </c>
       <c r="H36" s="8" t="inlineStr"/>
@@ -1938,17 +1938,17 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Maintain Copilot-side awareness of which cross-tenant / externally published agents can surface for the firm's users, sourced from the M365 admin center Agent registry and Integrated apps.</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Require documented admin approval before an externally published agent is made available to Copilot users; block end-user self-installation.</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Reconcile the Copilot-side approved list with FSI-AgentGov attestation and third-party review records quarterly; suspend Copilot availability of any agent whose AgentGov attestation has lapsed.</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -1980,17 +1980,17 @@
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Verify Unified Audit Log is enabled and actively recording events</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Upgrade to Audit (Premium) (E5 license tier) and create custom audit retention policies for Copilot record types — Audit (Premium) only extends the default retention to 1 year for Exchange/SharePoint/OneDrive/Entra audit records; `CopilotInteraction` and `CopilotAgentManagement` remain on the 180-day default until a custom policy is created</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Configure audit retention policies for 6+ years to help meet SEC Rule 17a-4(a) requirements using E5 Audit Premium with 10-year add-on retention or PAYG billing with governance controls</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr"/>
@@ -2022,17 +2022,17 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Create retention policies covering all Copilot content locations for a minimum of 3 years — required locations: Exchange Online (Copilot Chat substrate, Outlook drafts), Microsoft Copilot experiences (Copilot interaction history), SharePoint Online / All SharePoint Sites (team-shared files plus SharePoint Embedded containers used by Copilot Pages and Copilot Notebooks), OneDrive for Business (personal files and documents saved there, but not Pages storage), Teams Channel messages, Teams Chat messages, and Microsoft 365 Groups</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement differentiated retention periods based on the FSI retention matrix (3 years for communications, 6 years for financial records)</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Configure WORM-immutable retention for records subject to SEC Rule 17a-4(f) requirements — use `New-RetentionComplianceRule` with `-RetentionComplianceAction KeepAndDelete` to support immutable retain-then-delete behavior required for WORM compliance</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -2064,17 +2064,17 @@
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Verify Content search, eDiscovery (Standard), or eDiscovery (Premium) access based on the matter's required capabilities</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Deploy eDiscovery (Premium) capabilities for matters requiring custodian management, review sets, legal hold notices, analytics, or production sets</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Implement automated custodian identification and hold notification workflows in eDiscovery (Premium)</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr"/>
@@ -2106,17 +2106,17 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Create at least one Communication Compliance policy targeting Exchange and Teams locations</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Create separate policies for each communication type: regulatory compliance, conflict of interest, and custom firm-specific policies</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Deploy comprehensive policy coverage across all FINRA-regulated communication types</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -2148,17 +2148,17 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Document FINRA Rule 2210 (Communications with the Public) requirements in the firm's Copilot usage policies</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement a supervisory approval workflow that routes captured Copilot-drafted retail communications and risk-scored correspondence to registered principal review</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Implement mandatory pre-send supervisory review for all Copilot-drafted client communications by registered representatives</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr"/>
@@ -2190,17 +2190,17 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Update written supervisory procedures to address Copilot usage by associated persons</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Increase post-use review sampling rate to 25% of Copilot-assisted communications (FSI-recommended baseline); configure via CC policy &gt; Review percentage in the Purview portal</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Implement pre-send supervisory review for all Copilot-drafted client-facing communications (not just retail communications)</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -2232,17 +2232,17 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Map Copilot usage to existing regulatory reporting obligations</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Create automated report templates for each regulatory reporting obligation</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Implement automated evidence collection for regulatory report assembly (see Control 3.12)</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr"/>
@@ -2274,17 +2274,17 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Register Microsoft 365 Copilot in the enterprise model inventory with tier classification (Tier 3 for internal productivity, with documentation of the proportionality rationale for community banks per OCC Bulletin 2025-26). The AI inventory entry should include: tool name, version, purpose, business owner, deployment date, and risk classification</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Conduct use-case-specific output quality assessments quarterly</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Conduct annual comprehensive MRM assessment for Copilot aligned with SR 11-7 / OCC Bulletin 2011-12 expectations, including validation report focused on usage controls and output quality (not internal model architecture, which is Microsoft's responsibility as vendor)</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -2316,17 +2316,17 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Register Microsoft 365 Copilot in the enterprise model inventory as a generative AI system, cross-referencing the Control 3.8 inventory entry to avoid duplicate records.</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Define the validation scope for Copilot in writing, expressly limited to (a) usage controls and (b) output quality — not internal model architecture, which is Microsoft's responsibility as vendor.</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Conduct an annual comprehensive MRM assessment for Copilot that is cross-walked to all three frameworks (SR 11-7, NIST AI RMF 1.0, ISO/IEC 42001), with explicit gap analysis where the SR 26-2 exclusion creates open questions.</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr"/>
@@ -2358,17 +2358,17 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Establish an AI disclosure policy that addresses when and how Copilot usage is disclosed to clients</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement a marketing review process for all materials containing AI-related claims</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Implement automated detection of unauthorized AI claims in outbound communications</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -2400,17 +2400,17 @@
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Note the amended Reg S-P timeline: proposed March 2023, final rule adopted May 2024 (Release No. 34-100155), compliance deadline December 3, 2025 for larger firms and June 3, 2026 for smaller firms; key changes include expanded scope (investment advisers AND broker-dealers), mandatory written policies, expanded "customer information" definition, mandatory breach notification (≤30 days), and requirement for service providers to notify the institution within 72 hours of unauthorized access</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement sensitivity labels for NPI-containing content with DLP enforcement at the Copilot interaction layer</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Implement real-time NPI access monitoring for Copilot interactions using Microsoft Sentinel</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr"/>
@@ -2442,17 +2442,17 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Inventory all Copilot content locations and map them to 17a-3/4 record categories, including mobile access channels — key 17a-3 record types affected by Copilot: customer account records (Copilot-drafted account summaries, suitability notes), order tickets/blotter (Copilot-assisted trade order documentation), trade confirmations (Copilot-formatted confirmation drafts), written customer communications (any Copilot-drafted email via Outlook Copilot), agreements (Copilot-drafted advisory agreements), and supervisory records (Copilot-assisted supervisory review notes)</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement differentiated retention based on record category (3 years for communications, 6 years for financial records) — see 17a-3/4 retention period table above</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Implement WORM-compliant storage for Copilot records per SEC Rule 17a-4(f) — either via Option A (audit-trail alternative: Purview regulatory record labels + Preservation Lock with documented compliance analysis per Rule 17a-4(f)(2)(ii)(A)), or Option B (third-party WORM archival with vendor attestation)</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -2484,17 +2484,17 @@
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Define the evidence types required for each Copilot governance control</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Automate evidence collection where possible using PowerShell scripts and Purview API exports</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Implement fully automated evidence collection pipelines for operational evidence</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr"/>
@@ -2526,17 +2526,17 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Complete the FFIEC IT Handbook mapping for all deployed Copilot governance controls, focusing on the most relevant booklets:</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Align evidence collection (Control 3.12) with FFIEC examination expectations, mapping to key examination procedures:</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Commission independent FFIEC readiness assessment for Copilot governance, covering all relevant booklets (Information Security, AIO, Audit, Management) and supplemental guidance (OCC Bulletin 2025-26, SR 11-7)</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -2568,17 +2568,17 @@
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Establishes a default retention floor and basic lineage logging suitable for institutions whose Pages, Notebook, and Loop usage is primarily internal productivity rather than record-material work.</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Suitable for firms that use Pages and Notebooks for business-record-adjacent work (research, supervisory notes, product memos) and need lineage capture beyond the flat retention floor.</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Designed for broker-dealers, registered investment advisers, and other regulated firms where Copilot collaborative artifacts intersect with required records under SEC Rule 17a-4, FINRA Rule 4511(a), or SOX §§302/404 ICFR scope, and examination readiness is a regular operational expectation.</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr"/>
@@ -2610,17 +2610,17 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Assign Copilot administration to designated AI Administrators</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement segregation of duties so approval and implementation are not performed by the same person</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Require dual approval (technology + compliance) for new Copilot features, agent availability changes, or metered billing enablement</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -2652,17 +2652,17 @@
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Enforce `EnabledWithTranscript` via Teams meeting policy for all user groups with recordkeeping obligations — override the change announced September 2025 (MC1139493, effective late April 2026) that changed the global `-Copilot` default from `EnabledWithTranscript` to `Enabled`. FSI firms must explicitly set `-Copilot "EnabledWithTranscript"` on all regulated meeting policies to maintain transcript-coupled Copilot behavior required for record-keeping:</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Enforce `EnabledWithTranscript` for all users with Copilot licenses + configure auto-transcription for all scheduled meetings involving client discussions. Set additional meeting policy parameters for full coverage:</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Enforce `EnabledWithTranscript` + auto-transcription + auto-recording for all meetings involving regulated activities — verify enforcement across all assigned policies: `Get-CsTeamsMeetingPolicy | Select-Object Identity, Copilot, AllowTranscription, AllowCloudRecording`</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr"/>
@@ -2694,17 +2694,17 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Define which user groups have Copilot enabled for Teams Phone via calling policies — Copilot can run during PSTN and 1:1 VoIP calls, and AI-generated call summaries are produced when transcription is captured. The `-Copilot` parameter on `Set-CsTeamsCallingPolicy` controls call-Copilot availability (`Enabled` is the documented default; `EnabledWithTranscript` requires a started transcript before Copilot is offered; `Disabled` turns Copilot off for calls). For FSI recordkeeping, `EnabledWithTranscript` paired with `-AllowTranscriptionForCalling $true` is the recommended baseline so call Copilot only runs when a transcript is captured. Configure via Teams Admin Center &gt; Voice &gt; Calling policies:</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement supervisory review procedures for Copilot call summaries involving regulated activities</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Integrate Copilot call summaries into the firm's communication surveillance platform</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -2736,17 +2736,17 @@
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Configure Viva Insights minimum aggregation group size — default is 10; FSI recommended minimum is 10–25 for regulated departments. Differential privacy is applied to aggregated analytics. Portal: M365 Admin Center &gt; Viva &gt; Viva Insights &gt; Settings</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Exclude sensitive departments (legal, compliance, HR, internal audit) from Viva Insights organizational analytics — configure tenant admin exclusions to remove specific users (e.g., executives) from Insights analysis</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Include Viva Engage content in communication surveillance scope for communities discussing regulated topics — verify Communication Compliance policies reference "Viva Engage" location</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr"/>
@@ -2778,17 +2778,17 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Review M365 Copilot usage reports monthly</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Segment usage by department, risk tier, and billing model</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Include Copilot usage analytics in examination and SOX evidence packages where relevant</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -2820,17 +2820,17 @@
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Limit dashboard access to approved analysts</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Create a standardized Copilot impact summary for leadership</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Include impact measurement governance in examination and audit evidence where relevant</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr"/>
@@ -2862,17 +2862,17 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Review and configure Copilot feedback settings in M365 Admin Center</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Disable written (free-text) feedback for users in regulated roles (registered representatives, advisers, traders)</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Conduct annual privacy impact assessment specifically for Copilot feedback and telemetry data</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -2904,17 +2904,17 @@
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Maintain a current inventory of all Copilot licenses (type, quantity, assignment), including any active PAYG billing policies and the users or groups they cover. Track licenses by department:</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement usage-based license optimization with 60-day inactivity threshold</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Include Copilot license cost allocation in SOX internal control testing scope, including PAYG budget-notification authorization and escalation controls as part of IT general controls</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr"/>
@@ -2946,17 +2946,17 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Define AI incident classification taxonomy specific to Copilot</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement automated incident detection using DLP alerts, audit log monitoring, and anomaly detection</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Map Copilot incident types to specific regulatory notification requirements</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -2988,17 +2988,17 @@
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Conduct a Copilot dependency assessment to identify critical workflows</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Integrate Copilot service disruption scenarios into the organization's BCP</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Include Copilot BC/DR scenarios in annual BCP testing per FFIEC requirements</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr"/>
@@ -3030,17 +3030,17 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Enable the Microsoft 365 data connector in Sentinel</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Deploy all 5+ KQL detection queries listed in this control</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Implement correlation rules that combine Copilot events with other security signals (sign-in risk, DLP, insider risk)</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -3072,17 +3072,17 @@
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Assign a designated team member to monitor Microsoft Message Center for Copilot-related updates</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Implement a structured impact assessment for all Medium and High impact Copilot changes</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Integrate Copilot change management into the institution's formal ITGC change management program</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr"/>
@@ -3114,17 +3114,17 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Maintain a current inventory of plugins, connectors, and governed agents</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Review exception rate, adoption growth, and pending requests regularly</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Include high-risk extensibility and agent components in examination evidence packages</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -3156,17 +3156,17 @@
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Maintain Copilot-side visibility of published Copilot Studio agents available to the firm's Copilot users, from the M365 admin center Agent registry and Integrated apps.</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Require documented admin approval before a published agent is made available to Copilot users; block end-user self-installation.</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Reconcile the Copilot-side approved list with FSI-AgentGov lifecycle and publishing-approval records quarterly; suspend Copilot availability of any agent whose lifecycle evidence has lapsed.</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr"/>
@@ -3198,17 +3198,17 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Document the tenant's Cowork access posture: which users/groups have usage-based billing enabled, whether the discovery setting is on, and the approval basis for both decisions</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Manage usage-based billing scope, discovery, model toggles, browser-use toggle, and consumption limits through a documented change register</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Require dual approval (technology + compliance) before enabling usage-based billing, discovery, browser use, or the Anthropic/Fable model toggles for any regulated or client-facing population</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
@@ -3240,17 +3240,17 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>All Baseline requirements met (see control doc).</t>
+          <t>Document Frontier enrollment for the tenant and for admin accounts that will govern Scout</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>All Recommended requirements met (see control doc).</t>
+          <t>Manage Frontier scoping, endpoint policy, admin attestation, Microsoft 365 Copilot license assignment, and GitHub Copilot entitlement decisions through a documented change register with a named approver for each gate</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>All Regulated requirements met (see control doc).</t>
+          <t>Require dual approval (technology + compliance) before enabling Scout for any regulated or client-facing population</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: re-verify control 1.2 DSPM claims against current Microsoft Learn
Re-verifies the technical/product claims in
docs/controls/pillar-1-readiness/1.2-sharepoint-oversharing-detection.md
(last verified 2026-05-25) against live Microsoft Learn documentation and
the Microsoft 365 roadmap. Corrects drifted feature names, portal paths,
licensing SKUs, and documented product limits.

Technical-correctness only. No regulatory or compliance wording was added,
removed, or reinterpreted.

Regenerates the derived content graph and the two role templates that
reference control 1.2 so the mirrored Last Verified date and control text
stay consistent.

Refs judeper/OceanSquad#356

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -636,12 +636,12 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Addresses the most critical oversharing risks that could result in immediate regulatory exposure when Copilot is enabled. Shadow AI visibility is minimum viable governance for Copilot rollouts.</t>
+          <t>Addresses the most critical oversharing risks that could result in immediate regulatory exposure when Copilot is enabled. Visibility into unsanctioned AI apps is minimum viable governance for Copilot rollouts.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Provides ongoing oversharing governance with AI-specific visibility. Purview Posture Agent enables compliance teams to investigate data risks without requiring pre-defined SITs.</t>
+          <t>Provides ongoing oversharing governance with AI-specific visibility. The Data Security Posture Agent lets compliance teams investigate data risks without requiring pre-defined SITs.</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Extensibility Readiness (Graph Connectors, Plugins, Declarative Agents)</t>
+          <t>Extensibility Readiness (Copilot Connectors, Plugins, Declarative Agents)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: re-verify control 1.2 DSPM claims against current Microsoft Learn (#380)
Re-verifies the technical/product claims in
docs/controls/pillar-1-readiness/1.2-sharepoint-oversharing-detection.md
(last verified 2026-05-25) against live Microsoft Learn documentation and
the Microsoft 365 roadmap. Corrects drifted feature names, portal paths,
licensing SKUs, and documented product limits.

Technical-correctness only. No regulatory or compliance wording was added,
removed, or reinterpreted.

Regenerates the derived content graph and the two role templates that
reference control 1.2 so the mirrored Last Verified date and control text
stay consistent.

Refs judeper/OceanSquad#356

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/governance-maturity-dashboard.xlsx
+++ b/assessment/templates/governance-maturity-dashboard.xlsx
@@ -636,12 +636,12 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Addresses the most critical oversharing risks that could result in immediate regulatory exposure when Copilot is enabled. Shadow AI visibility is minimum viable governance for Copilot rollouts.</t>
+          <t>Addresses the most critical oversharing risks that could result in immediate regulatory exposure when Copilot is enabled. Visibility into unsanctioned AI apps is minimum viable governance for Copilot rollouts.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Provides ongoing oversharing governance with AI-specific visibility. Purview Posture Agent enables compliance teams to investigate data risks without requiring pre-defined SITs.</t>
+          <t>Provides ongoing oversharing governance with AI-specific visibility. The Data Security Posture Agent lets compliance teams investigate data risks without requiring pre-defined SITs.</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Extensibility Readiness (Graph Connectors, Plugins, Declarative Agents)</t>
+          <t>Extensibility Readiness (Copilot Connectors, Plugins, Declarative Agents)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">

</xml_diff>